<commit_message>
remove exposed sample answers and strengthen audits
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R5259a5fe61474b3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R45eb183bb57449de"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -459,18 +459,18 @@
     </x:row>
     <x:row r="20" ht="33" customHeight="1">
       <x:c r="A20" s="4" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>结果核对</x:v>
       </x:c>
       <x:c r="B20" s="4" t="str">
-        <x:v>源表保全、策略消费、冲销原因、SQLSTATE、RLS合同、角色探针和商户金额</x:v>
+        <x:v>来源表、策略消费、冲销原因、SQLSTATE、RLS合同、角色访问和商户金额能够互相追溯</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="33" customHeight="1">
       <x:c r="A21" s="4" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
+        <x:v>实现自由度</x:v>
       </x:c>
       <x:c r="B21" s="4" t="str">
-        <x:v>CTE拆分、别名、索引名、注释、缩进、内部查询顺序、CSV必要引号和LF或CRLF行尾</x:v>
+        <x:v>CTE拆分、别名、索引名、注释、缩进和内部查询顺序可以不同，CSV允许必要引号及LF或CRLF行尾</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>